<commit_message>
Updated BOM and added a generic, more descriptive version
</commit_message>
<xml_diff>
--- a/hardware/WindRose_V01_0B_BOM.xlsx
+++ b/hardware/WindRose_V01_0B_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandro\Documents\ProjetoMarilia\HW_V01_0B\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a645505eb1d0d43f/Desktop/HW_WR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42F3810C-6FAF-4B67-A020-A0AD8F0DD67A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{439C7065-0F4D-43D9-8F73-4A89C639EB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" BOM Template" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Designator</t>
     <phoneticPr fontId="18" type="noConversion"/>
@@ -98,9 +98,6 @@
     <t>R2</t>
   </si>
   <si>
-    <t>https://statics3.seeedstudio.com/fusion/opl/datasheet/301010207.pdf</t>
-  </si>
-  <si>
     <t>https://statics3.seeedstudio.com/fusion/opl/datasheet/301010047.pdf</t>
   </si>
   <si>
@@ -120,6 +117,12 @@
   </si>
   <si>
     <t>AMS1117-5.0</t>
+  </si>
+  <si>
+    <t>https://file.elecfans.com/web2/M00/5A/77/poYBAGLrqhuANnZQAA8p9tNjF34381.pdf</t>
+  </si>
+  <si>
+    <t>RT0603DRD07220RL</t>
   </si>
 </sst>
 </file>
@@ -736,14 +739,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -753,9 +756,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42">
@@ -824,9 +824,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -864,7 +864,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -970,7 +970,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1112,7 +1112,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1121,25 +1121,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E38"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.59765625" style="1" customWidth="1"/>
     <col min="2" max="2" width="43.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="115.625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="7.3984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="119.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="19.5" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="7"/>
+      <c r="E5" s="6"/>
     </row>
     <row r="6" spans="1:5" ht="19.5" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -1219,13 +1219,13 @@
         <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="19.5" customHeight="1">
@@ -1246,14 +1246,14 @@
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="3">
-        <v>301010207</v>
+      <c r="B9" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="C9" s="3">
         <v>1</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="19.5" customHeight="1">
@@ -1267,7 +1267,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.5" customHeight="1">
@@ -1281,7 +1281,7 @@
         <v>5</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="19.5" customHeight="1">
@@ -1289,7 +1289,7 @@
         <v>17</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
@@ -1300,7 +1300,7 @@
     </row>
     <row r="13" spans="1:5" ht="19.5" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="3">
         <v>306030002</v>
@@ -1309,94 +1309,94 @@
         <v>1</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="16.5">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.8">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" ht="16.5">
+    <row r="17" spans="1:4" ht="16.8">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" ht="16.5">
+    <row r="18" spans="1:4" ht="16.8">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" ht="16.5">
+    <row r="19" spans="1:4" ht="16.8">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" ht="16.5">
+    <row r="20" spans="1:4" ht="16.8">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" ht="16.5">
+    <row r="21" spans="1:4" ht="16.8">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" ht="16.5">
+    <row r="22" spans="1:4" ht="16.8">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" ht="16.5">
+    <row r="23" spans="1:4" ht="16.8">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="1:4" ht="16.5">
+    <row r="24" spans="1:4" ht="16.8">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="4"/>
     </row>
-    <row r="25" spans="1:4" ht="16.5">
+    <row r="25" spans="1:4" ht="16.8">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="1:4" ht="16.5">
+    <row r="26" spans="1:4" ht="16.8">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="1:4" ht="16.5">
+    <row r="27" spans="1:4" ht="16.8">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="16.5">
+    <row r="28" spans="1:4" ht="16.8">
       <c r="A28" s="2"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="1:4" ht="16.5">
+    <row r="29" spans="1:4" ht="16.8">
       <c r="A29" s="2"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="1:4" ht="16.5">
+    <row r="30" spans="1:4" ht="16.8">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="1:4" ht="16.5">
+    <row r="31" spans="1:4" ht="16.8">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="3"/>

</xml_diff>